<commit_message>
Add teacher subject sorting and fix date template
</commit_message>
<xml_diff>
--- a/static/templates/Mau_import_hoc_sinh.xlsx
+++ b/static/templates/Mau_import_hoc_sinh.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh sách học sinh" sheetId="1" r:id="R463b476b51d648cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh sách học sinh" sheetId="1" r:id="R65c3443387f0484e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1220,6 +1220,18 @@
       <x:c r="B200" s="14"/>
       <x:c r="D200" s="16"/>
     </x:row>
+    <x:row r="201">
+      <x:c r="D201" s="16"/>
+    </x:row>
+    <x:row r="202">
+      <x:c r="D202" s="16"/>
+    </x:row>
+    <x:row r="203">
+      <x:c r="D203" s="16"/>
+    </x:row>
+    <x:row r="204">
+      <x:c r="D204" s="16"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>

</xml_diff>